<commit_message>
fix : scrolling and login
</commit_message>
<xml_diff>
--- a/attached_assets/list_books.xlsx
+++ b/attached_assets/list_books.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\b_outside\a_intesa_global_technology\Storify\Storify-Insights\Storify-Insights\attached_assets\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EDC4B103-EB33-406B-B9A3-3881A4C712FA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CFEE881D-7CF6-459E-A842-AD682CC2F94C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="30936" windowHeight="16776" xr2:uid="{61CDC90C-EC06-4A7D-B103-BEBAB272D490}"/>
+    <workbookView xWindow="15264" yWindow="0" windowWidth="15552" windowHeight="16656" xr2:uid="{61CDC90C-EC06-4A7D-B103-BEBAB272D490}"/>
   </bookViews>
   <sheets>
     <sheet name="list_books" sheetId="1" r:id="rId1"/>
@@ -1771,7 +1771,7 @@
       <family val="2"/>
     </font>
   </fonts>
-  <fills count="33">
+  <fills count="34">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -1951,6 +1951,12 @@
         <bgColor indexed="65"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="5" tint="0.59999389629810485"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
   </fills>
   <borders count="10">
     <border>
@@ -2112,9 +2118,10 @@
     <xf numFmtId="0" fontId="1" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="1" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="7" fillId="3" borderId="0" xfId="7"/>
+    <xf numFmtId="0" fontId="0" fillId="33" borderId="0" xfId="0" applyFill="1"/>
   </cellXfs>
   <cellStyles count="42">
     <cellStyle name="20% - Accent1" xfId="19" builtinId="30" customBuiltin="1"/>
@@ -4231,7 +4238,7 @@
       </c>
     </row>
     <row r="103" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A103" t="s">
+      <c r="A103" s="2" t="s">
         <v>298</v>
       </c>
       <c r="B103" t="s">
@@ -4673,7 +4680,7 @@
       </c>
     </row>
     <row r="129" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A129" t="s">
+      <c r="A129" s="2" t="s">
         <v>328</v>
       </c>
       <c r="B129" t="s">
@@ -4826,7 +4833,7 @@
       </c>
     </row>
     <row r="138" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A138" t="s">
+      <c r="A138" s="2" t="s">
         <v>403</v>
       </c>
       <c r="B138" t="s">
@@ -4860,7 +4867,7 @@
       </c>
     </row>
     <row r="140" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A140" t="s">
+      <c r="A140" s="2" t="s">
         <v>343</v>
       </c>
       <c r="B140" t="s">
@@ -4877,7 +4884,7 @@
       </c>
     </row>
     <row r="141" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A141" t="s">
+      <c r="A141" s="2" t="s">
         <v>340</v>
       </c>
       <c r="B141" t="s">
@@ -5129,7 +5136,7 @@
       </c>
     </row>
     <row r="156" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A156" t="s">
+      <c r="A156" s="2" t="s">
         <v>530</v>
       </c>
       <c r="B156" t="s">
@@ -5605,7 +5612,7 @@
       </c>
     </row>
     <row r="184" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A184" t="s">
+      <c r="A184" s="2" t="s">
         <v>417</v>
       </c>
       <c r="B184" t="s">
@@ -5639,7 +5646,7 @@
       </c>
     </row>
     <row r="186" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A186" t="s">
+      <c r="A186" s="2" t="s">
         <v>421</v>
       </c>
       <c r="B186" t="s">
@@ -5979,7 +5986,7 @@
       </c>
     </row>
     <row r="206" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A206" t="s">
+      <c r="A206" s="2" t="s">
         <v>444</v>
       </c>
       <c r="B206" t="s">
@@ -6166,7 +6173,7 @@
       </c>
     </row>
     <row r="217" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A217" t="s">
+      <c r="A217" s="2" t="s">
         <v>457</v>
       </c>
       <c r="B217" t="s">
@@ -6251,7 +6258,7 @@
       </c>
     </row>
     <row r="222" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A222" t="s">
+      <c r="A222" s="2" t="s">
         <v>474</v>
       </c>
       <c r="B222" t="s">
@@ -6302,7 +6309,7 @@
       </c>
     </row>
     <row r="225" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A225" t="s">
+      <c r="A225" s="2" t="s">
         <v>481</v>
       </c>
       <c r="B225" t="s">

</xml_diff>